<commit_message>
wärmeerzeuger und beedarf mit hinzugefügt
</commit_message>
<xml_diff>
--- a/data/Optimierungsgrößen.xlsx
+++ b/data/Optimierungsgrößen.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HansisRasanterRaser\Desktop\UNI\000_DA\git\knEBiD\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A475DA3-B18E-4D39-8ED4-8FAE401F4457}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B892557-3042-4278-883C-6282382D4541}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1078,7 +1078,7 @@
         <v>4400</v>
       </c>
       <c r="F10" s="1">
-        <v>9999</v>
+        <v>99999</v>
       </c>
       <c r="G10" s="1">
         <v>999</v>
@@ -1104,7 +1104,7 @@
         <v>359</v>
       </c>
       <c r="F11" s="1">
-        <v>999</v>
+        <v>99999</v>
       </c>
       <c r="G11" s="1">
         <v>999</v>
@@ -1130,7 +1130,7 @@
         <v>100</v>
       </c>
       <c r="F12" s="1">
-        <v>999</v>
+        <v>99999</v>
       </c>
       <c r="G12" s="1">
         <v>999</v>
@@ -1156,7 +1156,7 @@
         <v>100</v>
       </c>
       <c r="F13" s="1">
-        <v>999</v>
+        <v>99999</v>
       </c>
       <c r="G13" s="1">
         <v>999</v>

</xml_diff>